<commit_message>
Estabilizar scraper sync y dashboard support
</commit_message>
<xml_diff>
--- a/data/incremental/incremental_01_las_condes_manual.xlsx
+++ b/data/incremental/incremental_01_las_condes_manual.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restaurantes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Restaurantes'!$A$1:$AG$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Restaurantes'!$A$1:$AG$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG27"/>
+  <dimension ref="A1:AG31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
@@ -460,7 +460,7 @@
     <col width="15" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="17" customWidth="1" min="32" max="32"/>
-    <col width="22" customWidth="1" min="33" max="33"/>
+    <col width="42" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,52 +633,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>La Cabrera Chile Isidora</t>
+          <t>LA NOSTRA CASA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>283</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 3275, 7550129 Las Condes, Región Metropolitana</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>9 3452 4440</t>
-        </is>
-      </c>
+          <t>Av. Las Condes 6901, 7560846 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://lacabrerachile.cl/</t>
+          <t>https://www.instagram.com/lanostracasa.trattoria</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restaurante italiano</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/La+Cabrera+Chile+Isidora/data=!4m7!3m6!1s0x9662cf1a85a95ee5:0x1afc90f8f5200406!8m2!3d-33.4146907!4d-70.5966256!16s%2Fg%2F11pzx6mqls!19sChIJ5V6phRrPYpYRBgQg9fiQ_Bo?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/LA+NOSTRA+CASA/data=!4m7!3m6!1s0x9662cf262070b505:0x8ccb48b41941f271!8m2!3d-33.4062332!4d-70.5595921!16s%2Fg%2F11yp4kxwld!19sChIJBbVwICbPYpYRcfJBGbRIy4w?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>-33.4146907</t>
+          <t>-33.4062332</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-70.5966256</t>
+          <t>-70.5595921</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -703,12 +699,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Completo</t>
+          <t>Sin teléfono</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -731,12 +727,16 @@
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Sin teléfono visible</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Diablo Vino y Fuego Restaurante</t>
+          <t>La Cabrera Chile Isidora</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -746,22 +746,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>65</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mercado Urbano Tobalaba (MUT - Av. Apoquindo 2730, 5to Piso, 7550179 Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 3275, 7550129 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9 5006 3696</t>
+          <t>9 3452 4440</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://diablorestaurant.com/</t>
+          <t>https://lacabrerachile.cl/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -771,17 +771,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Diablo+Vino+y+Fuego+Restaurante/data=!4m7!3m6!1s0x9662cf000e465ddb:0x6db641c2529150bd!8m2!3d-33.4176518!4d-70.6013263!16s%2Fg%2F11ybgm1n6y!19sChIJ211GDgDPYpYRvVCRUsJBtm0?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/La+Cabrera+Chile+Isidora/data=!4m7!3m6!1s0x9662cf1a85a95ee5:0x1afc90f8f5200406!8m2!3d-33.4146907!4d-70.5966256!16s%2Fg%2F11pzx6mqls!19sChIJ5V6phRrPYpYRBgQg9fiQ_Bo?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>-33.4176518</t>
+          <t>-33.4146907</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>-70.6013263</t>
+          <t>-70.5966256</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -839,52 +839,52 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kató Tasty Caos</t>
+          <t>Diablo Vino y Fuego Restaurante</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>731</t>
+          <t>97</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 3275, local 2, 7550129 Las Condes, Región Metropolitana</t>
+          <t>Mercado Urbano Tobalaba (MUT - Av. Apoquindo 2730, 5to Piso, 7550179 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9 7663 1330</t>
+          <t>9 5006 3696</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://katotastycaos.cl/</t>
+          <t>https://diablorestaurant.com/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Restaurante de cocina panasiática</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Kat%C3%B3+Tasty+Caos/@-33.4146907,-70.5966256,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf43fd970a8b:0xc8f06bea80827d12!8m2!3d-33.4146907!4d-70.5966256!16s%2Fg%2F11mkhstszp?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Diablo+Vino+y+Fuego+Restaurante/data=!4m7!3m6!1s0x9662cf000e465ddb:0x6db641c2529150bd!8m2!3d-33.4176518!4d-70.6013263!16s%2Fg%2F11ybgm1n6y!19sChIJ211GDgDPYpYRvVCRUsJBtm0?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>-33.4146907</t>
+          <t>-33.4176518</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>-70.5966256</t>
+          <t>-70.6013263</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -942,52 +942,52 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hijo del Sol Las condes</t>
+          <t>Kató Tasty Caos</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>731</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 3215, 7550083 Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 3275, local 2, 7550129 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9 9770 2222</t>
+          <t>9 7663 1330</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/hijodelsol.santiago/</t>
+          <t>https://katotastycaos.cl/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Restaurante peruano</t>
+          <t>Restaurante de cocina panasiática</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Hijo+del+Sol+Las+condes/@-33.4146584,-70.5968579,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf00105e07af:0x8803bd86a3a14b42!8m2!3d-33.4146584!4d-70.5968579!16s%2Fg%2F11vxm2gzdv?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Kat%C3%B3+Tasty+Caos/data=!4m7!3m6!1s0x9662cf43fd970a8b:0xc8f06bea80827d12!8m2!3d-33.4146907!4d-70.5966256!16s%2Fg%2F11mkhstszp!19sChIJiwqX_UPPYpYREn2CgOpr8Mg?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>-33.4146584</t>
+          <t>-33.4146907</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-70.5968579</t>
+          <t>-70.5966256</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1045,52 +1045,52 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Raffaella Cucina Napoletana</t>
+          <t>Hijo del Sol Las condes</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>944</t>
+          <t>309</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ntra. Sra. del Rosario 21, 7560763 Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 3215, 7550083 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9 4018 6723</t>
+          <t>9 9770 2222</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>http://www.raffaellacucina.cl/</t>
+          <t>https://www.instagram.com/hijodelsol.santiago/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Restaurante italiano</t>
+          <t>Restaurante peruano</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Raffaella+Cucina+Napoletana/data=!4m7!3m6!1s0x9662cff574ae6adb:0x32b078a303f2f8ec!8m2!3d-33.4063143!4d-70.5612246!16s%2Fg%2F11s1v1pqdl!19sChIJ22qudPXPYpYR7PjyA6N4sDI?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Hijo+del+Sol+Las+condes/data=!4m7!3m6!1s0x9662cf00105e07af:0x8803bd86a3a14b42!8m2!3d-33.4146584!4d-70.5968579!16s%2Fg%2F11vxm2gzdv!19sChIJrwdeEADPYpYRQkuho4a9A4g?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>-33.4063143</t>
+          <t>-33.4146584</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-70.5612246</t>
+          <t>-70.5968579</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1148,52 +1148,52 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Restoran Pinpilinpausha</t>
+          <t>Raffaella Cucina Napoletana</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>945</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 2900, 7550033 Las Condes, Región Metropolitana</t>
+          <t>Ntra. Sra. del Rosario 21, 7560763 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(2) 3275 4303</t>
+          <t>9 4018 6723</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>http://www.pinpilinpausha.cl/</t>
+          <t>http://www.raffaellacucina.cl/</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Restaurante de cocina española</t>
+          <t>Restaurante italiano</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Restoran+Pinpilinpausha/@-33.4137939,-70.6017388,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf41a61d994b:0xf33a25474c22bc39!8m2!3d-33.4137939!4d-70.6017388!16s%2Fg%2F1tg7t6hy?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Raffaella+Cucina+Napoletana/data=!4m7!3m6!1s0x9662cff574ae6adb:0x32b078a303f2f8ec!8m2!3d-33.4063143!4d-70.5612246!16s%2Fg%2F11s1v1pqdl!19sChIJ22qudPXPYpYR7PjyA6N4sDI?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-33.4137939</t>
+          <t>-33.4063143</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-70.6017388</t>
+          <t>-70.5612246</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>98</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Lumi%C3%A9re+Bistr%C3%B3+Restaurante/@-33.4124303,-70.5787114,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf95117ec80d:0xc51680b1d08a9f02!8m2!3d-33.4124303!4d-70.5787114!16s%2Fg%2F11x318xkp_?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Lumi%C3%A9re+Bistr%C3%B3+Restaurante/data=!4m7!3m6!1s0x9662cf95117ec80d:0xc51680b1d08a9f02!8m2!3d-33.4124303!4d-70.5787114!16s%2Fg%2F11x318xkp_!19sChIJDch-EZXPYpYRAp-K0LGAFsU?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1354,52 +1354,52 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Chilmex</t>
+          <t>Restoran Pinpilinpausha</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>80</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Gral. Carol Urzúa 7065, 7560796 Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 2900, 7550033 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(2) 2886 0775</t>
+          <t>(2) 3275 4303</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>http://chilmex.cl/</t>
+          <t>http://www.pinpilinpausha.cl/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restaurante de cocina española</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Chilmex/data=!4m7!3m6!1s0x9662cf8fc31ea7a5:0x64a78c382180dc11!8m2!3d-33.4054821!4d-70.5572147!16s%2Fg%2F11fkblc7fj!19sChIJpacew4_PYpYREdyAITiMp2Q?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Restoran+Pinpilinpausha/data=!4m7!3m6!1s0x9662cf41a61d994b:0xf33a25474c22bc39!8m2!3d-33.4137939!4d-70.6017388!16s%2Fg%2F1tg7t6hy!19sChIJS5kdpkHPYpYRObwiTEclOvM?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>-33.4054821</t>
+          <t>-33.4137939</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-70.5572147</t>
+          <t>-70.6017388</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1457,52 +1457,48 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Trattoria Rita Parque Arauco</t>
+          <t>UDON Alto Las Condes</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>254</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Av. Pdte. Kennedy 5413, Local 369, 7550000 Las Condes, Región Metropolitana</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>(2) 2656 7014</t>
-        </is>
-      </c>
+          <t>Av. Pdte. Kennedy 9001, 7591567 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>http://www.rita.cl/</t>
+          <t>https://www.udon.cl/restaurante/alto-las-condes/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Restaurante italiano</t>
+          <t>Restaurante asiático</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Trattoria+Rita+Parque+Arauco/@-33.4020735,-70.5786617,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf385855f3b5:0x725ed6a2b990a40a!8m2!3d-33.4020735!4d-70.5786617!16s%2Fg%2F11mhj__345?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/UDON+Alto+Las+Condes/data=!4m7!3m6!1s0x9662cf001f20f919:0x1f51acb385c12dc0!8m2!3d-33.3908304!4d-70.5472432!16s%2Fg%2F11myt8k__d!19sChIJGfkgHwDPYpYRwC3BhbOsUR8?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-33.4020735</t>
+          <t>-33.3908304</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-70.5786617</t>
+          <t>-70.5472432</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1527,12 +1523,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Completo</t>
+          <t>Sin teléfono</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1555,35 +1551,43 @@
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Sin teléfono visible</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Toni Lautaro</t>
+          <t>Chilmex</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>58</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Avenida Apoquindo 2730, MUT 4to piso, Las Condes, Región Metropolitana</t>
+          <t>Gral. Carol Urzúa 7065, 7560796 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9 7963 7286</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>(2) 2886 0775</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>http://chilmex.cl/</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Restaurante</t>
@@ -1591,17 +1595,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Toni+Lautaro/data=!4m7!3m6!1s0x9662cf59110ee7d5:0xd5f5da5ab1f5418f!8m2!3d-33.4176518!4d-70.6013263!16s%2Fg%2F11w3b3g_7j!19sChIJ1ecOEVnPYpYRj0H1sVra9dU?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Chilmex/data=!4m7!3m6!1s0x9662cf8fc31ea7a5:0x64a78c382180dc11!8m2!3d-33.4054821!4d-70.5572147!16s%2Fg%2F11fkblc7fj!19sChIJpacew4_PYpYREdyAITiMp2Q?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-33.4176518</t>
+          <t>-33.4054821</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-70.6013263</t>
+          <t>-70.5572147</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1626,12 +1630,12 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Completo</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1659,48 +1663,52 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Almuerzo las condes</t>
+          <t>Trattoria Rita Parque Arauco</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>García Pica 6784, 7560260 Las Condes, Región Metropolitana</t>
+          <t>Av. Pdte. Kennedy 5413, Local 369, 7550000 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9 6231 8141</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>(2) 2656 7014</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>http://www.rita.cl/</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restaurante italiano</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Almuerzo+las+condes/data=!4m7!3m6!1s0x9662cfcfd3976653:0x8e38586ff678a61e!8m2!3d-33.3995587!4d-70.5622255!16s%2Fg%2F11h01flnvq!19sChIJU2aX08_PYpYRHqZ49m9YOI4?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Trattoria+Rita+Parque+Arauco/data=!4m7!3m6!1s0x9662cf385855f3b5:0x725ed6a2b990a40a!8m2!3d-33.4020735!4d-70.5786617!16s%2Fg%2F11mhj__345!19sChIJtfNVWDjPYpYRCqSQuaLWXnI?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>-33.3995587</t>
+          <t>-33.4020735</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-70.5622255</t>
+          <t>-70.5786617</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1725,12 +1733,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Completo</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1758,52 +1766,52 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bali Hai Chile</t>
+          <t>La Fattoria</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>162</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Av. Cristóbal Colón 5146, 7580214 Las Condes, Región Metropolitana</t>
+          <t>Av. Apoquindo 5680, 7560943 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(2) 3375 9696</t>
+          <t>(2) 2377 6000</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.balihai.cl/</t>
+          <t>https://fattoriarestaurant.simplybook.me/</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Restaurante polinesio</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Bali+Hai+Chile/@-33.4184462,-70.5716536,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cee3b7afead9:0x5b5b5dfaec2585db!8m2!3d-33.4184462!4d-70.5716536!16s%2Fg%2F1hjgt49yn?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/La+Fattoria/data=!4m7!3m6!1s0x9662cede5273ffff:0x97ad4366a3600d8d!8m2!3d-33.409551!4d-70.571085!16s%2Fg%2F11hdy27qz2!19sChIJ__9zUt7OYpYRjQ1go2ZDrZc?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>-33.4184462</t>
+          <t>-33.409551</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>-70.5716536</t>
+          <t>-70.571085</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1828,7 +1836,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1861,52 +1869,48 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Koychi Korean Street Food</t>
+          <t>Toni Lautaro</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>77</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Av. Pdte. Kennedy 5413, 7550000 Las Condes, Región Metropolitana</t>
+          <t>Avenida Apoquindo 2730, MUT 4to piso, Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>9 9393 3419</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>https://www.koychi.cl/</t>
-        </is>
-      </c>
+          <t>9 7963 7286</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Restaurante coreano</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Koychi+Korean+Street+Food/@-33.402211,-70.5769511,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cfaa23f923f3:0xaaf956e9dce8757a!8m2!3d-33.402211!4d-70.5769511!16s%2Fg%2F11vkggpt__?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Toni+Lautaro/data=!4m7!3m6!1s0x9662cf59110ee7d5:0xd5f5da5ab1f5418f!8m2!3d-33.4176518!4d-70.6013263!16s%2Fg%2F11w3b3g_7j!19sChIJ1ecOEVnPYpYRj0H1sVra9dU?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>-33.402211</t>
+          <t>-33.4176518</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>-70.5769511</t>
+          <t>-70.6013263</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1931,12 +1935,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Completo</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1964,52 +1968,52 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Restorant el Castillo</t>
+          <t>Piano Gourmet Restaurante y Café</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>143</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Av. Apoquindo 7092, 7571726 Las Condes, Región Metropolitana</t>
+          <t>Av. Padre Hurtado Nte 77, 7591575 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9 5036 3284</t>
+          <t>9 9128 7273</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://instagram.com/el.castillo.restaurante?igshid=YWJhMjlhZTc=</t>
+          <t>http://www.pianogourmet.cl/</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Cafetería</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Restorant+el+Castillo/data=!4m7!3m6!1s0x9662cec1f1885d91:0xa5a6f52ad52d8dab!8m2!3d-33.407713!4d-70.5556445!16s%2Fg%2F1tv25bnz!19sChIJkV2I8cHOYpYRq40t1Sr1pqU?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Piano+Gourmet+Restaurante+y+Caf%C3%A9/data=!4m7!3m6!1s0x9662cfc9db72f817:0x449f3256a68a0e89!8m2!3d-33.393639!4d-70.545679!16s%2Fg%2F11whmx2ln1!19sChIJF_hy28nPYpYRiQ6KplYyn0Q?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>-33.407713</t>
+          <t>-33.393639</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-70.5556445</t>
+          <t>-70.545679</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2034,7 +2038,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2044,7 +2048,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R15" t="inlineStr"/>
@@ -2062,57 +2066,61 @@
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Revisar: parece cafeteria; Revisar: parece cafe</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Don Carlos</t>
+          <t>Bali Hai Chile</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 2895, 7550101 Las Condes, Región Metropolitana</t>
+          <t>Av. Cristóbal Colón 5146, 7580214 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>9 4850 0864</t>
+          <t>(2) 3375 9696</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.doncarloscarneyvino.cl/</t>
+          <t>https://www.balihai.cl/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restaurante polinesio</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Don+Carlos/data=!4m7!3m6!1s0x9662cf41a61379ad:0xeb84305be2c0d72e!8m2!3d-33.414149!4d-70.601774!16s%2Fg%2F1tdw027v!19sChIJrXkTpkHPYpYRLtfA4lswhOs?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Bali+Hai+Chile/data=!4m7!3m6!1s0x9662cee3b7afead9:0x5b5b5dfaec2585db!8m2!3d-33.4184462!4d-70.5716536!16s%2Fg%2F1hjgt49yn!19sChIJ2eqvt-POYpYR24Ul7PpdW1s?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>-33.414149</t>
+          <t>-33.4184462</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-70.601774</t>
+          <t>-70.5716536</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2137,7 +2145,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2170,34 +2178,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Route 66</t>
+          <t>Almuerzo las condes</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 2960, 7550059 Las Condes, Región Metropolitana</t>
+          <t>García Pica 6784, 7560260 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>(2) 3266 9954</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>http://www.route66.cl/</t>
-        </is>
-      </c>
+          <t>9 6231 8141</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Restaurante</t>
@@ -2205,17 +2209,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Route+66/data=!4m7!3m6!1s0x9662cf405ad73ffb:0xee029d663f1a73e7!8m2!3d-33.4139825!4d-70.5999351!16s%2Fg%2F11dymmkn9y!19sChIJ-z_XWkDPYpYR53MaP2adAu4?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Almuerzo+las+condes/data=!4m7!3m6!1s0x9662cfcfd3976653:0x8e38586ff678a61e!8m2!3d-33.3995587!4d-70.5622255!16s%2Fg%2F11h01flnvq!19sChIJU2aX08_PYpYRHqZ49m9YOI4?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>-33.4139825</t>
+          <t>-33.3995587</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-70.5999351</t>
+          <t>-70.5622255</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2240,12 +2244,12 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Completo</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2273,7 +2277,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Happening</t>
+          <t>Restorant el Castillo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2283,22 +2287,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>509</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Av. Apoquindo 3090, 7550312 Las Condes, Región Metropolitana</t>
+          <t>Av. Apoquindo 7092, 7571726 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(2) 2362 1092</t>
+          <t>9 5036 3284</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>http://www.happening.cl/</t>
+          <t>https://instagram.com/el.castillo.restaurante?igshid=YWJhMjlhZTc=</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2308,17 +2312,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Happening/data=!4m7!3m6!1s0x9662cf154a3d39f5:0x1037462ca6ea9cf5!8m2!3d-33.416711!4d-70.5976522!16s%2Fg%2F1ts_7tfh!19sChIJ9Tk9ShXPYpYR9ZzqpixGNxA?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Restorant+el+Castillo/data=!4m7!3m6!1s0x9662cec1f1885d91:0xa5a6f52ad52d8dab!8m2!3d-33.407713!4d-70.5556445!16s%2Fg%2F1tv25bnz!19sChIJkV2I8cHOYpYRq40t1Sr1pqU?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-33.416711</t>
+          <t>-33.407713</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-70.5976522</t>
+          <t>-70.5556445</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2343,7 +2347,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2376,52 +2380,52 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aligot restaurant</t>
+          <t>Koychi Korean Street Food</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 2890, 7550033 Las Condes, Región Metropolitana</t>
+          <t>Av. Pdte. Kennedy 5413, 7550000 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(41) 324 8475</t>
+          <t>9 9393 3419</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://toto.menu/aligot?s=googlemaps</t>
+          <t>https://www.koychi.cl/</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restaurante coreano</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Aligot+restaurant/@-33.413808,-70.6019947,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cfac435bdaad:0x7ed19e2ff27dfbdf!8m2!3d-33.413808!4d-70.6019947!16s%2Fg%2F11h3swvrz_?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Koychi+Korean+Street+Food/data=!4m7!3m6!1s0x9662cfaa23f923f3:0xaaf956e9dce8757a!8m2!3d-33.402211!4d-70.5769511!16s%2Fg%2F11vkggpt__!19sChIJ8yP5I6rPYpYRenXo3OlW-ao?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-33.413808</t>
+          <t>-33.402211</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>-70.6019947</t>
+          <t>-70.5769511</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2446,7 +2450,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2479,7 +2483,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>La Flaca, Cocinería Chilena</t>
+          <t>Don Carlos</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2489,22 +2493,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>69</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Av. Apoquindo 2730, Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 2895, 7550101 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>(2) 2437 6668</t>
+          <t>9 4850 0864</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://laflaca.cl/</t>
+          <t>https://www.doncarloscarneyvino.cl/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2514,17 +2518,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/La+Flaca,+Cociner%C3%ADa+Chilena/data=!4m7!3m6!1s0x9662c53939e3eebb:0xdc2e7676299d3b56!8m2!3d-33.4177122!4d-70.6013629!16s%2Fg%2F11c3tj92p4!19sChIJu-7jOTnFYpYRVjudKXZ2Ltw?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Don+Carlos/data=!4m7!3m6!1s0x9662cf41a61379ad:0xeb84305be2c0d72e!8m2!3d-33.414149!4d-70.601774!16s%2Fg%2F1tdw027v!19sChIJrXkTpkHPYpYRLtfA4lswhOs?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>-33.4177122</t>
+          <t>-33.414149</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>-70.6013629</t>
+          <t>-70.601774</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2549,7 +2553,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2582,32 +2586,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Chilenazo Las Condes</t>
+          <t>Route 66</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Av. Apoquindo 6226, 7561215 Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 2960, 7550059 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(2) 2201 7162</t>
+          <t>(2) 3266 9954</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.chilenazorestaurant.cl/Locales/las-condes/</t>
+          <t>http://www.route66.cl/</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2617,17 +2621,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Chilenazo+Las+Condes/data=!4m7!3m6!1s0x9662ceddb1a2b61f:0x2405a15bc5dbaf28!8m2!3d-33.4082051!4d-70.5663157!16s%2Fg%2F1td4frpk!19sChIJH7aisd3OYpYRKK_bxVuhBSQ?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Route+66/data=!4m7!3m6!1s0x9662cf405ad73ffb:0xee029d663f1a73e7!8m2!3d-33.4139825!4d-70.5999351!16s%2Fg%2F11dymmkn9y!19sChIJ-z_XWkDPYpYR53MaP2adAu4?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-33.4082051</t>
+          <t>-33.4139825</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-70.5663157</t>
+          <t>-70.5999351</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2652,7 +2656,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2685,7 +2689,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>La Perla del Pacífico</t>
+          <t>Nowa´s Cantina</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2695,22 +2699,18 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>90</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Av. Pdte. Kennedy 5413, 372 A, 7550000 Las Condes, Región Metropolitana</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>(2) 2656 7013</t>
-        </is>
-      </c>
+          <t>Pdte. Riesco 5330, Local 103, 7560996 Santiago, Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>http://www.laperladelpacifico.cl/</t>
+          <t>http://www.nowascantina.cl/</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2720,17 +2720,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/La+Perla+del+Pac%C3%ADfico/@-33.4022776,-70.5771918,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf3a8a5dcfad:0xf2ae9b520b7f2c33!8m2!3d-33.4022776!4d-70.5771918!16s%2Fg%2F11cjg5r3fw?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Nowa%C2%B4s+Cantina/data=!4m7!3m6!1s0x9662cfaeb22d158b:0x64a2d89a3e3c9c03!8m2!3d-33.4033611!4d-70.5751261!16s%2Fg%2F11shs_28h_!19sChIJixUtsq7PYpYRA5w8PprYomQ?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-33.4022776</t>
+          <t>-33.4033611</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-70.5771918</t>
+          <t>-70.5751261</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2755,12 +2755,12 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Completo</t>
+          <t>Sin teléfono</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2783,33 +2783,41 @@
       <c r="AD22" t="inlineStr"/>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>Sin teléfono visible</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Nowa´s Cantina</t>
+          <t>Estró Santiago</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>528</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Pdte. Riesco 5330, Local 103, 7560996 Santiago, Las Condes, Región Metropolitana</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t>El Alcalde 15, 7550655 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>(2) 2470 8585</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>http://www.nowascantina.cl/</t>
+          <t>http://www.instagram.com/estrosantiago</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2819,17 +2827,17 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Nowa%C2%B4s+Cantina/@-33.4033611,-70.5751261,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cfaeb22d158b:0x64a2d89a3e3c9c03!8m2!3d-33.4033611!4d-70.5751261!16s%2Fg%2F11shs_28h_?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Estr%C3%B3+Santiago/data=!4m7!3m6!1s0x9662cf157bee637f:0x73257e215251e871!8m2!3d-33.4158983!4d-70.5952355!16s%2Fg%2F11c542nyfq!19sChIJf2PuexXPYpYRcehRUiF-JXM?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>-33.4033611</t>
+          <t>-33.4158983</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-70.5751261</t>
+          <t>-70.5952355</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2854,12 +2862,12 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Sin teléfono</t>
+          <t>Completo</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2882,41 +2890,37 @@
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>Sin teléfono visible</t>
-        </is>
-      </c>
+      <c r="AG23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Margó Isidora Goyenechea</t>
+          <t>Aligot restaurant</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Isidora Goyenechea 3000, S-101, Santiago, Las Condes, Región Metropolitana</t>
+          <t>Isidora Goyenechea 2890, 7550033 Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>(2) 2385 0178</t>
+          <t>(41) 324 8475</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>http://margo.cl/</t>
+          <t>https://toto.menu/aligot?s=googlemaps</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2926,17 +2930,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Marg%C3%B3+Isidora+Goyenechea/@-33.4141182,-70.598816,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cf406edb17b7:0xbfbe9d33a013c8e7!8m2!3d-33.4141182!4d-70.598816!16s%2Fg%2F11hdc40fpl?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Aligot+restaurant/data=!4m7!3m6!1s0x9662cfac435bdaad:0x7ed19e2ff27dfbdf!8m2!3d-33.413808!4d-70.6019947!16s%2Fg%2F11h3swvrz_!19sChIJrdpbQ6zPYpYR3_t98i-e0X4?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>-33.4141182</t>
+          <t>-33.413808</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>-70.598816</t>
+          <t>-70.6019947</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2961,7 +2965,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2994,48 +2998,52 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Black Chicken</t>
+          <t>Mr. Dumpling Chile</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Cerro El Plomo 5931, 7550000 Las Condes, Región Metropolitana</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>Encomenderos 210, 7550152 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>9 4267 3634</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>http://www.blackchicken.cl/</t>
+          <t>http://www.instagram.com/mrdumplingcl</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Restaurante especializado en pollo</t>
+          <t>Restaurante asiático</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Black+Chicken/@-33.4045086,-70.5704691,17z/data=!3m1!4b1!4m6!3m5!1s0x9662cb39191c9253:0xbe925edbd3daa79c!8m2!3d-33.4045086!4d-70.5704691!16s%2Fg%2F11l_dz254l?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Mr.+Dumpling+Chile/data=!4m7!3m6!1s0x9662cfebddb23037:0x4fc60f30b484c467!8m2!3d-33.4164598!4d-70.6027326!16s%2Fg%2F11k5540ldp!19sChIJNzCy3evPYpYRZ8SEtDAPxk8?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>-33.4045086</t>
+          <t>-33.4164598</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>-70.5704691</t>
+          <t>-70.6027326</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3060,12 +3068,12 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Sin teléfono</t>
+          <t>Completo</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3088,41 +3096,37 @@
       <c r="AD25" t="inlineStr"/>
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>Sin teléfono visible</t>
-        </is>
-      </c>
+      <c r="AG25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Puerto Del Alto</t>
+          <t>La Flaca, Cocinería Chilena</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mirador del Alto - Av. Pdte. Kennedy 9001, Local 3235, 7591567 Las Condes, Región Metropolitana</t>
+          <t>Av. Apoquindo 2730, Las Condes, Región Metropolitana</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>(2) 2656 7012</t>
+          <t>(2) 2437 6668</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>http://www.puertodelalto.cl/</t>
+          <t>https://laflaca.cl/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3132,17 +3136,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Puerto+Del+Alto/@-33.3901082,-70.546859,17z/data=!3m1!4b1!4m6!3m5!1s0x9662ceb4360029b3:0xa5e9a254925036d5!8m2!3d-33.3901082!4d-70.546859!16s%2Fg%2F11f10bk9c0?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUyMC4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/La+Flaca,+Cociner%C3%ADa+Chilena/data=!4m7!3m6!1s0x9662c53939e3eebb:0xdc2e7676299d3b56!8m2!3d-33.4177122!4d-70.6013629!16s%2Fg%2F11c3tj92p4!19sChIJu-7jOTnFYpYRVjudKXZ2Ltw?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>-33.3901082</t>
+          <t>-33.4177122</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>-70.546859</t>
+          <t>-70.6013629</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3167,7 +3171,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3200,48 +3204,48 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Barra Chalaca - Alto Las Condes</t>
+          <t>Olivia Trattoria</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>314</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Av. Pdte. Kennedy 9001, 7591567 Las Condes, Región Metropolitana</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>https://barrachalaca.cl/</t>
-        </is>
-      </c>
+          <t>O'connell 165, Piso -1, 7560811 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>9 9569 7805</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Restaurante italiano</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Barra+Chalaca+-+Alto+Las+Condes/data=!4m7!3m6!1s0x9662cfe010e7fa67:0x74cccfebd6fa726f!8m2!3d-33.391703!4d-70.5459846!16s%2Fg%2F11w48hsbgx!19sChIJZ_rnEODPYpYRb3L61uvPzHQ?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+          <t>https://www.google.com/maps/place/Olivia+Trattoria/data=!4m7!3m6!1s0x9662cfffd614f85b:0x4207972b4cd99e5c!8m2!3d-33.4072818!4d-70.5685356!16s%2Fg%2F11vq56ch5q!19sChIJW_gU1v_PYpYRXJ7ZTCuXB0I?authuser=0&amp;hl=es-419&amp;rclk=1</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>-33.391703</t>
+          <t>-33.4072818</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>-70.5459846</t>
+          <t>-70.5685356</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3266,12 +3270,12 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Sin teléfono</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -3294,14 +3298,422 @@
       <c r="AD27" t="inlineStr"/>
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr">
-        <is>
-          <t>Sin teléfono visible</t>
-        </is>
-      </c>
+      <c r="AG27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TPM BAR</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>402</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Av. Las Condes 6766, 7550000 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>(2) 2833 2889</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>http://www.tpmbar.cl/</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Bar restaurante</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/TPM+BAR/data=!4m7!3m6!1s0x9662cf4a95155799:0x42753b0ac97319c4!8m2!3d-33.4064945!4d-70.5607861!16s%2Fg%2F11sczxm5dx!19sChIJmVcVlUrPYpYRxBlzyQo7dUI?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>-33.4064945</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>-70.5607861</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Las Condes</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Google Maps web scraping con Playwright</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>IL Pazzo</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Alonso de Córdova 5320, 7550000 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>9 3030 5510</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>http://www.ilpazzo.cl/</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/IL+Pazzo/data=!4m7!3m6!1s0x9662cf9e39fec851:0x76495c6d5c926973!8m2!3d-33.406343!4d-70.5742281!16s%2Fg%2F11m_nwrtnq!19sChIJUcj-OZ7PYpYRc2mSXG1cSXY?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>-33.406343</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>-70.5742281</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Las Condes</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Google Maps web scraping con Playwright</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Happening</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Av. Apoquindo 3090, 7550312 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>(2) 2362 1092</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>http://www.happening.cl/</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Happening/data=!4m7!3m6!1s0x9662cf154a3d39f5:0x1037462ca6ea9cf5!8m2!3d-33.416711!4d-70.5976522!16s%2Fg%2F1ts_7tfh!19sChIJ9Tk9ShXPYpYR9ZzqpixGNxA?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>-33.416711</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>-70.5976522</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Las Condes</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Google Maps web scraping con Playwright</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+      <c r="AG30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Chilenazo Las Condes</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Av. Apoquindo 6226, 7561215 Las Condes, Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>(2) 2201 7162</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.chilenazorestaurant.cl/Locales/las-condes/</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Chilenazo+Las+Condes/data=!4m7!3m6!1s0x9662ceddb1a2b61f:0x2405a15bc5dbaf28!8m2!3d-33.4082051!4d-70.5663157!16s%2Fg%2F1td4frpk!19sChIJH7aisd3OYpYRKK_bxVuhBSQ?authuser=0&amp;hl=es-419&amp;rclk=1</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>-33.4082051</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>-70.5663157</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Las Condes</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Google Maps web scraping con Playwright</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG27"/>
+  <autoFilter ref="A1:AG31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>